<commit_message>
Add tenders and small purchases sheet to SALT_CLOTHES_KONKURS_1210.xlsx
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JQLkwre52iMXL7eAYSL71v
</commit_message>
<xml_diff>
--- a/SALT_CLOTHES_KONKURS_1210.xlsx
+++ b/SALT_CLOTHES_KONKURS_1210.xlsx
@@ -9,10 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Соль" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Одежда" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Тендеры и малые закупки" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Соль'!$A$1:$R$2</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Одежда'!$A$1:$R$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Тендеры и малые закупки'!$A$1:$R$7</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1411,4 +1413,509 @@
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:R7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="17" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="9" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>№</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Тип</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Статус</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Номер закупки</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Предмет</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Заказчик</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Регион</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Закон</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Способ</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Площадка</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>НМЦК, ₽</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Окончание подачи</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Только СМП</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Обеспечение заявки</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Обеспечение контракта</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>Аванс</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>Ссылка</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Примечание</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Спецодежда / СИЗ</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Актуален</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>100920595126100116</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Поставка средств индивидуальной защиты для работников ГАУК ЛО "Международный центр реставрации в целях выполнения государственного задания на 2026 г. ГАУК ЛО "Международный центр реставрации" часть 1</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Государственное автономное учреждение Культуры Ленинградской обл. «Международный Центр Реставрации»</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>47 Ленинградская область</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Малые закупки</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Малая закупка</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>ЕАТ (Березка)</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>517291.1</v>
+      </c>
+      <c r="L2" s="5" t="n">
+        <v>46314.375</v>
+      </c>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="n">
+        <v>25864.56</v>
+      </c>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Сыпучие/хозтовары (соль может быть в спецификации — проверить)</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Актуален</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>3764771</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Закупка в 2026 году хозяйственных товаров для нужд дошкольного отделения МБОУ Часцовской СОШ</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Муниципальное бюджетное общеобразовательное учреждение Часцовская СОШ</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>50 Московская область</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Малые закупки</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Малая закупка</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Электронный магазин Московской области</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>69996</v>
+      </c>
+      <c r="L3" s="5" t="n">
+        <v>46311.61805555555</v>
+      </c>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Сыпучие/хозтовары (соль может быть в спецификации — проверить)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Актуален</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>10743414</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Закупка в 2026 году хозяйственных товаров для нужд дошкольного отделения МБОУ Часцовской СОШ</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Муниципальное бюджетное общеобразовательное учреждение Часцовская СОШ</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>50 Московская область</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Малые закупки</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Малая закупка</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>РТС-тендер</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>69996</v>
+      </c>
+      <c r="L4" s="5" t="n">
+        <v>46311.61805555555</v>
+      </c>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Сыпучие/хозтовары (соль может быть в спецификации — проверить)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Актуален</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>6241366</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Закупка в 2026 году хозяйственных товаров для нужд дошкольного отделения МБОУ Часцовской СОШ</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Муниципальное бюджетное общеобразовательное учреждение Часцовская СОШ</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>50 Московская область</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Коммерческие</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Тендер</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Портал поставщиков</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>69996</v>
+      </c>
+      <c r="L5" s="5" t="n">
+        <v>46311.61805555555</v>
+      </c>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Спецодежда / СИЗ</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Актуален</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>383-467</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Закупка специальной одежды и СИЗ на склад Томилино</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>АО «Кюхенлэнд Хоум Рус»</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>23 Краснодарский край</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Коммерческие</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Тендер</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Bidzaar</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="n"/>
+      <c r="L6" s="5" t="n">
+        <v>46311.625</v>
+      </c>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>НМЦК не указана — цену запрашивать</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Спецодежда / СИЗ</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Актуален</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>372-446</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Приобретение специальной одежды, специальной обуви, СИЗ</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>ООО «Благо-Армавир»</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>23 Краснодарский край</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Коммерческие</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Тендер</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Bidzaar</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="n"/>
+      <c r="L7" s="5" t="n">
+        <v>46314.70833333334</v>
+      </c>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>НМЦК не указана — цену запрашивать</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:R7"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>